<commit_message>
Sumar resumen para la Evaluacion 1 de GDSI y resumenes simples de Redes, CdD y GDSI; actualizar calendarios (CdD: parcial al 29/10; GDSI: cronograma v0.5, recuperatorio al 16/11) y rehacer los planes de estudio
</commit_message>
<xml_diff>
--- a/Materias/Ciencia de Datos/Calendario 2do 2026.xlsx
+++ b/Materias/Ciencia de Datos/Calendario 2do 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>Cronograma - 2026 2C
 Ciencia de Datos - TA047
@@ -31,22 +31,91 @@
     <t>Práctica (Jueves)</t>
   </si>
   <si>
-    <t xml:space="preserve">Presentación de la materia.
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Presentación de la materia.
 Visualización de datos.
 </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1thITCAk3lT4H2a9Z9o7eEMSBxY_L52PE/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1FifyUeNa2ogPCiH77RT_4ZE0XGMXLz0_/view</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Introducción a Colab y maquinas Jupyter
+    <t>Introducción a Colab y maquinas Jupyter
 Pandas - Librerías de visualización.
-</t>
-  </si>
-  <si>
-    <t>Introducción a la ciencia de datos.
-Métodos de regresión
-Métricas</t>
+Sin grabación</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Introducción a la ciencia de datos.
+Métodos de regresión
+Métricas
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1wIvWCdAYIshUCfArXji1RU3EiG527jAJ/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1EFgcv5vlYQnazORuclFw4SpmJAvRIqYJ/view</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
       <t xml:space="preserve">Métodos de regresión
 Métricas
 </t>
@@ -55,49 +124,97 @@
       <rPr>
         <rFont val="Calibri"/>
         <b/>
-        <color theme="1"/>
         <sz val="14.0"/>
       </rPr>
-      <t>Fecha Límite Grupos TP1 - Presentación TP1</t>
+      <t xml:space="preserve">Fecha Límite Grupos TP1 - Presentación TP1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1jxRMBG8JlJ-jY8JFfwuihMusSTVvTEmF/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Métodos de clasificación
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Métodos de clasificación
 Métodos de agrupamiento (clustering)
 Métricas
 </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1rsYTJr8fofht6yTCCqrDy519uUzRp-7l/view</t>
+    </r>
   </si>
   <si>
-    <t>Métodos de clasificación
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Métodos de clasificación
 Métodos de agrupamiento (clustering)
-Metricas</t>
+Metricas
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1dXOSl-uy3aAKkRgvfv7YNHG1OAimI_44/view</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Ingeniería de características
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Ingeniería de características
 </t>
-  </si>
-  <si>
-    <t>Árboles de decisión
-Ensambles: Random Forest / XgBoost</t>
-  </si>
-  <si>
-    <t>k-nearest neighbors algorithm
-Support Vector Machines (SVM)
-Ensambles Híbridos</t>
-  </si>
-  <si>
-    <t>Redes neuronales artificiales superficiales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redes neuronales artificiales superficiales
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/drive/folders/1TRnn6Eux6YCRaAeYYOubq0wqynC6ZMSp?usp=sharing</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
-  </si>
-  <si>
-    <t>Reduccion de la dimensionalidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reduccion de la dimensionalidad
-</t>
+    </r>
   </si>
   <si>
     <r>
@@ -106,7 +223,301 @@
         <color rgb="FF000000"/>
         <sz val="14.0"/>
       </rPr>
-      <t xml:space="preserve">Consultas parcial
+      <t xml:space="preserve">Ingeniería de características
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1z-QaZtYiK-cVEIfWZ3MOMYaGls3zpIWY/view</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Árboles de decisión
+Ensambles: Random Forest / XgBoost
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1e1yiRZvY3LNgSPRknd6368b2Y1qz9dFb/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1oK87UIXlWG8lcZMp5a2sEk6zdsLv5QTp/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Árboles de decisión
+Ensambles: Random Forest / XgBoost
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/drive/folders/1zUm6V3f36h7b4ow3SuRJBMSbgB6iHMf0?usp=sharing</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/drive/folders/1DA7KfglfseQuU5-ZNFyuigOPqjLPyVjz?usp=drive_link</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">k-nearest neighbors algorithm
+Support Vector Machines (SVM)
+Ensambles Híbridos
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://youtu.be/3EYL8bhQsbU</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://youtu.be/ACbBEaGSn3I</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">k-nearest neighbors algorithm
+Support Vector Machines (SVM)
+Ensambles Híbridos
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/drive/folders/1YdbhP2GiYSvjniSzvIQTwIWh_FvGD7tu?usp=sharing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Redes neuronales artificiales superficiales
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1guv1nMx19fkARmBZyBHScrJAVgXCtSD2/view?usp=sharing</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1pyOjPYjKsBW2XbqlBPSuDk2nAJFQAlE5/view?usp=sharing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Redes neuronales artificiales superficiales
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/drive/folders/1Q31R4rLXmQVphkAPXVBHjZAcqYnKSa6y?usp=sharing</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Reduccion de la dimensionalidad
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1yIe3GvIjpda0MCslK1EnDQM9cC9DE5rR/view</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/1ptuEDI1g8snlCx8ioi6xM5CsBAUYlnmt/view</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Reduccion de la dimensionalidad
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="14.0"/>
+        <u/>
+      </rPr>
+      <t>https://drive.google.com/file/d/17yE27RhjzSva7zgNDl6PHP31zz76Iq-t/view</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF000000"/>
+        <sz val="14.0"/>
+      </rPr>
+      <t xml:space="preserve">Procesamiento de lenguaje natural (PLN)
 </t>
     </r>
     <r>
@@ -121,38 +532,20 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Parcial (Presencial)
-</t>
+    <t>-- paro --</t>
   </si>
   <si>
     <t xml:space="preserve">Exposición TP1
 </t>
   </si>
   <si>
+    <t>Procesamiento de lenguaje natural (PLN)</t>
+  </si>
+  <si>
     <t>Exposición TP1</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="14.0"/>
-      </rPr>
-      <t>Procesamiento de lenguaje natural (PLN)</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="14.0"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>Procesamiento de lenguaje natural (PLN)</t>
+    <t>Parcial (Presencial)</t>
   </si>
   <si>
     <t>Introducción a las redes profundas</t>
@@ -194,7 +587,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="17">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -232,7 +625,42 @@
     </font>
     <font>
       <sz val="14.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="14.0"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14.0"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -479,13 +907,13 @@
     <xf borderId="11" fillId="5" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="12" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="12" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="11" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="12" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -494,43 +922,34 @@
     <xf borderId="11" fillId="4" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="11" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf borderId="11" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="11" fillId="5" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="11" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="11" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="6" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="6" fontId="15" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="11" fillId="6" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="11" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="6" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="11" fillId="6" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="12" fillId="6" fontId="14" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="11" fillId="6" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="11" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="11" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="11" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="12" fillId="6" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="12" fillId="6" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="12" fillId="6" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="11" fillId="4" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -539,7 +958,16 @@
     <xf borderId="11" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="4" fontId="14" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="13" fillId="2" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -897,15 +1325,15 @@
         <f t="shared" si="1"/>
         <v>46273</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="19" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="17">
         <f t="shared" si="2"/>
         <v>46275</v>
       </c>
-      <c r="F7" s="24" t="s">
-        <v>11</v>
+      <c r="F7" s="23" t="s">
+        <v>12</v>
       </c>
       <c r="G7" s="4"/>
     </row>
@@ -920,19 +1348,19 @@
         <f t="shared" si="1"/>
         <v>46280</v>
       </c>
-      <c r="D8" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="24">
+      <c r="D8" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="25">
         <f t="shared" si="2"/>
         <v>46282</v>
       </c>
-      <c r="F8" s="26" t="s">
-        <v>12</v>
+      <c r="F8" s="23" t="s">
+        <v>14</v>
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" ht="76.5" customHeight="1">
+    <row r="9" ht="96.75" customHeight="1">
       <c r="A9" s="13">
         <v>6.0</v>
       </c>
@@ -943,15 +1371,15 @@
         <f t="shared" si="1"/>
         <v>46287</v>
       </c>
-      <c r="D9" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="24">
+      <c r="D9" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="25">
         <f t="shared" si="2"/>
         <v>46289</v>
       </c>
-      <c r="F9" s="26" t="s">
-        <v>13</v>
+      <c r="F9" s="23" t="s">
+        <v>16</v>
       </c>
       <c r="G9" s="4"/>
     </row>
@@ -966,19 +1394,19 @@
         <f t="shared" si="1"/>
         <v>46294</v>
       </c>
-      <c r="D10" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="24">
+      <c r="D10" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="25">
         <f t="shared" si="2"/>
         <v>46296</v>
       </c>
-      <c r="F10" s="26" t="s">
-        <v>15</v>
+      <c r="F10" s="23" t="s">
+        <v>18</v>
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" ht="37.5" customHeight="1">
+    <row r="11" ht="83.25" customHeight="1">
       <c r="A11" s="13">
         <v>8.0</v>
       </c>
@@ -989,15 +1417,15 @@
         <f t="shared" si="1"/>
         <v>46301</v>
       </c>
-      <c r="D11" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="24">
+      <c r="D11" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="25">
         <f t="shared" si="2"/>
         <v>46303</v>
       </c>
-      <c r="F11" s="26" t="s">
-        <v>17</v>
+      <c r="F11" s="23" t="s">
+        <v>20</v>
       </c>
       <c r="G11" s="4"/>
     </row>
@@ -1010,15 +1438,15 @@
         <f t="shared" si="1"/>
         <v>46308</v>
       </c>
-      <c r="D12" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="27">
+      <c r="D12" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="22">
         <f t="shared" si="2"/>
         <v>46310</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -1033,14 +1461,14 @@
         <v>46315</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="30">
+        <v>23</v>
+      </c>
+      <c r="E13" s="17">
         <f t="shared" si="2"/>
         <v>46317</v>
       </c>
-      <c r="F13" s="28" t="s">
-        <v>21</v>
+      <c r="F13" s="30" t="s">
+        <v>24</v>
       </c>
       <c r="G13" s="4"/>
     </row>
@@ -1051,19 +1479,19 @@
       <c r="B14" s="14">
         <v>44865.0</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="29">
         <f t="shared" si="1"/>
         <v>46322</v>
       </c>
-      <c r="D14" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="E14" s="17">
+      <c r="D14" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="31">
         <f t="shared" si="2"/>
         <v>46324</v>
       </c>
-      <c r="F14" s="33" t="s">
-        <v>23</v>
+      <c r="F14" s="32" t="s">
+        <v>26</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -1074,19 +1502,19 @@
       <c r="B15" s="14">
         <v>44872.0</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="33">
         <f t="shared" si="1"/>
         <v>46329</v>
       </c>
-      <c r="D15" s="32" t="s">
-        <v>24</v>
+      <c r="D15" s="34" t="s">
+        <v>27</v>
       </c>
       <c r="E15" s="17">
         <f t="shared" si="2"/>
         <v>46331</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G15" s="4"/>
     </row>
@@ -1097,19 +1525,19 @@
       <c r="B16" s="14">
         <v>44879.0</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="33">
         <f t="shared" si="1"/>
         <v>46336</v>
       </c>
-      <c r="D16" s="32" t="s">
-        <v>26</v>
+      <c r="D16" s="34" t="s">
+        <v>29</v>
       </c>
       <c r="E16" s="17">
         <f t="shared" si="2"/>
         <v>46338</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -1120,19 +1548,19 @@
       <c r="B17" s="14">
         <v>44886.0</v>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="33">
         <f t="shared" si="1"/>
         <v>46343</v>
       </c>
-      <c r="D17" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="34">
+      <c r="D17" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="31">
         <f t="shared" si="2"/>
         <v>46345</v>
       </c>
-      <c r="F17" s="35" t="s">
-        <v>28</v>
+      <c r="F17" s="32" t="s">
+        <v>31</v>
       </c>
       <c r="G17" s="4"/>
     </row>
@@ -1143,19 +1571,19 @@
       <c r="B18" s="14">
         <v>44893.0</v>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="33">
         <f t="shared" si="1"/>
         <v>46350</v>
       </c>
-      <c r="D18" s="32" t="s">
-        <v>29</v>
+      <c r="D18" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="E18" s="17">
         <f>C18+2</f>
         <v>46352</v>
       </c>
-      <c r="F18" s="33" t="s">
-        <v>30</v>
+      <c r="F18" s="30" t="s">
+        <v>33</v>
       </c>
       <c r="G18" s="4"/>
     </row>
@@ -1166,25 +1594,25 @@
       <c r="B19" s="14">
         <v>44900.0</v>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="35">
         <f t="shared" si="1"/>
         <v>46357</v>
       </c>
-      <c r="D19" s="37" t="s">
-        <v>31</v>
+      <c r="D19" s="36" t="s">
+        <v>34</v>
       </c>
       <c r="E19" s="17">
         <f>C19+2</f>
         <v>46359</v>
       </c>
-      <c r="F19" s="26" t="s">
-        <v>32</v>
+      <c r="F19" s="37" t="s">
+        <v>35</v>
       </c>
       <c r="G19" s="4"/>
     </row>
     <row r="20">
       <c r="A20" s="38" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B20" s="39"/>
       <c r="C20" s="39"/>
@@ -8030,6 +8458,23 @@
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="A20:F21"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="D4"/>
+    <hyperlink r:id="rId2" ref="D5"/>
+    <hyperlink r:id="rId3" ref="F5"/>
+    <hyperlink r:id="rId4" ref="D6"/>
+    <hyperlink r:id="rId5" ref="F6"/>
+    <hyperlink r:id="rId6" ref="D7"/>
+    <hyperlink r:id="rId7" ref="F7"/>
+    <hyperlink r:id="rId8" ref="D8"/>
+    <hyperlink r:id="rId9" ref="F8"/>
+    <hyperlink r:id="rId10" ref="D9"/>
+    <hyperlink r:id="rId11" ref="F9"/>
+    <hyperlink r:id="rId12" ref="D10"/>
+    <hyperlink r:id="rId13" ref="F10"/>
+    <hyperlink r:id="rId14" ref="D11"/>
+    <hyperlink r:id="rId15" ref="F11"/>
+  </hyperlinks>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>